<commit_message>
WEEK 2 and WEEK 3
</commit_message>
<xml_diff>
--- a/Batch 2/Week 3/sample_data/sample_data.xlsx
+++ b/Batch 2/Week 3/sample_data/sample_data.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Project Antigravity</t>
+          <t>Project RAG Chatbot</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Project Antigravity</t>
+          <t>Project RAG Chatbot</t>
         </is>
       </c>
     </row>

</xml_diff>